<commit_message>
Updated pre-week 3 exercise 1A
</commit_message>
<xml_diff>
--- a/pre-week-3/homework1_exerciseAI.xlsx
+++ b/pre-week-3/homework1_exerciseAI.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30606"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3ED0CFFE-5170-4A21-9529-051051700F63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{14EA5222-6ACF-4A3B-BC00-0F728F35EC1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -213,8 +213,8 @@
     <c:plotArea>
       <c:layout/>
       <c:barChart>
-        <c:barDir val="bar"/>
-        <c:grouping val="percentStacked"/>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
         <c:varyColors val="0"/>
         <c:ser>
           <c:idx val="0"/>
@@ -331,126 +331,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-C3E6-4C2D-8FA9-D8D9818DF330}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:ser>
-          <c:idx val="1"/>
-          <c:order val="1"/>
-          <c:tx>
-            <c:strRef>
-              <c:f>Sheet1!$C$1</c:f>
-              <c:strCache>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>Average Rating</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:tx>
-          <c:spPr>
-            <a:solidFill>
-              <a:schemeClr val="accent2"/>
-            </a:solidFill>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:invertIfNegative val="0"/>
-          <c:cat>
-            <c:strRef>
-              <c:f>Sheet1!$A$2:$A$13</c:f>
-              <c:strCache>
-                <c:ptCount val="12"/>
-                <c:pt idx="0">
-                  <c:v>Python Programming</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>Data Analytics</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>Web Devlopment</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>Cybersecurity</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>Cloud Computing</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>Java Programming</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>Machine Learning</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>Database Management</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>Business Analytics</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>Excel Fundamentals</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>Project Management</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>Network Security</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>Sheet1!$C$2:$C$13</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="12"/>
-                <c:pt idx="0">
-                  <c:v>4.8</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>4.7</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>4.5</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>4.5999999999999996</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>4.4000000000000004</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>4.3</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>4.9000000000000004</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>4.2</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>4.5</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>4.7</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>4.0999999999999996</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>3.8</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:val>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-C3E6-4C2D-8FA9-D8D9818DF330}"/>
+              <c16:uniqueId val="{00000000-5069-468A-83E0-C37CDB804E1A}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -462,18 +343,18 @@
           <c:showPercent val="0"/>
           <c:showBubbleSize val="0"/>
         </c:dLbls>
-        <c:gapWidth val="150"/>
-        <c:overlap val="100"/>
-        <c:axId val="1038164487"/>
-        <c:axId val="1038166535"/>
+        <c:gapWidth val="219"/>
+        <c:overlap val="-27"/>
+        <c:axId val="1316570631"/>
+        <c:axId val="1316572679"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="1038164487"/>
+        <c:axId val="1316570631"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
         <c:delete val="0"/>
-        <c:axPos val="l"/>
+        <c:axPos val="b"/>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
@@ -511,7 +392,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1038166535"/>
+        <c:crossAx val="1316572679"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -519,12 +400,12 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1038166535"/>
+        <c:axId val="1316572679"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
         <c:delete val="0"/>
-        <c:axPos val="b"/>
+        <c:axPos val="l"/>
         <c:majorGridlines>
           <c:spPr>
             <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
@@ -539,7 +420,7 @@
             <a:effectLst/>
           </c:spPr>
         </c:majorGridlines>
-        <c:numFmt formatCode="0%" sourceLinked="1"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -570,7 +451,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1038164487"/>
+        <c:crossAx val="1316570631"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -691,7 +572,7 @@
 </file>
 
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="297">
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="201">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
     <cs:fillRef idx="0"/>
@@ -895,23 +776,22 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
+      <a:schemeClr val="dk1"/>
     </cs:fontRef>
     <cs:spPr>
       <a:solidFill>
         <a:schemeClr val="dk1">
-          <a:lumMod val="75000"/>
-          <a:lumOff val="25000"/>
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
         </a:schemeClr>
       </a:solidFill>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:ln w="9525">
         <a:solidFill>
           <a:schemeClr val="tx1">
             <a:lumMod val="65000"/>
             <a:lumOff val="35000"/>
           </a:schemeClr>
         </a:solidFill>
-        <a:round/>
       </a:ln>
     </cs:spPr>
   </cs:downBar>
@@ -1016,8 +896,8 @@
       <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
         <a:solidFill>
           <a:schemeClr val="tx1">
-            <a:lumMod val="50000"/>
-            <a:lumOff val="50000"/>
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
           </a:schemeClr>
         </a:solidFill>
         <a:round/>
@@ -1149,20 +1029,19 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
+      <a:schemeClr val="dk1"/>
     </cs:fontRef>
     <cs:spPr>
       <a:solidFill>
         <a:schemeClr val="lt1"/>
       </a:solidFill>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:ln w="9525">
         <a:solidFill>
           <a:schemeClr val="tx1">
-            <a:lumMod val="65000"/>
-            <a:lumOff val="35000"/>
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
           </a:schemeClr>
         </a:solidFill>
-        <a:round/>
       </a:ln>
     </cs:spPr>
   </cs:upBar>
@@ -1200,22 +1079,22 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>552450</xdr:colOff>
+      <xdr:colOff>504825</xdr:colOff>
       <xdr:row>1</xdr:row>
-      <xdr:rowOff>133350</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>247650</xdr:colOff>
-      <xdr:row>16</xdr:row>
-      <xdr:rowOff>19050</xdr:rowOff>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>352425</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="2" name="Chart 1">
+        <xdr:cNvPr id="3" name="Chart 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{435A6682-DE89-CCC3-166D-26EB01D50789}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6F058974-FAD2-17CA-F47F-35544AA3EECB}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>

</xml_diff>